<commit_message>
Update student ID for น.ส.อัชฌา จันตะคุณ to 6730108592
</commit_message>
<xml_diff>
--- a/มอบตัว69 (1).xlsx
+++ b/มอบตัว69 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\โครงการทิศทางเฟรชชี่ The Freshy Bearing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5164E63-EEF2-4620-B4D2-2E56E6F4BF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5816151-4A51-460C-B9C5-9D4C7702F684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108104,7 +108104,7 @@
         <v>9285</v>
       </c>
       <c r="G51" s="5">
-        <v>6730108582</v>
+        <v>6730108592</v>
       </c>
     </row>
     <row r="52" spans="1:7">

</xml_diff>

<commit_message>
Update Mr. Thanawat Tacha-ampai's ticket display to replace STAFF with ADVISOR
</commit_message>
<xml_diff>
--- a/มอบตัว69 (1).xlsx
+++ b/มอบตัว69 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\โครงการทิศทางเฟรชชี่ The Freshy Bearing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD580808-14E5-4DE4-96B6-2D74DCB677DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A1CC330-97D1-44A3-87DC-C9FC7528F090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28020,10 +28020,10 @@
     <t xml:space="preserve">นายธนวัฒน์ เตชะอำไพ </t>
   </si>
   <si>
-    <t>SAB69</t>
-  </si>
-  <si>
     <t>รหัสการค้นชื่อ</t>
+  </si>
+  <si>
+    <t>sab69</t>
   </si>
 </sst>
 </file>
@@ -108724,10 +108724,10 @@
         <v>9325</v>
       </c>
       <c r="F112" s="4" t="s">
+        <v>9327</v>
+      </c>
+      <c r="G112" s="4" t="s">
         <v>9328</v>
-      </c>
-      <c r="G112" s="4" t="s">
-        <v>9327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update student database: add 1 new student (Tariswan Saowarakkun) stably without changing existing 3,452 assignments
</commit_message>
<xml_diff>
--- a/มอบตัว69 (1).xlsx
+++ b/มอบตัว69 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\โครงการทิศทางเฟรชชี่ The Freshy Bearing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B942E0-0007-4D41-BAFD-B4FE8A341817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37EC04E0-8EC1-43AF-ADB9-020B959F7671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24321" uniqueCount="9326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24327" uniqueCount="9328">
   <si>
     <t>id_student</t>
   </si>
@@ -28016,6 +28016,12 @@
   </si>
   <si>
     <t>Organizer THE FTESHY BEARING   รองนายกฝ่ายบริหาร   อนุกรรมการเหรัญญิก   ที่ปรึกษาส่วนตัวนายกองค์การบริหาร องค์การนิสิต</t>
+  </si>
+  <si>
+    <t>ธฤษวรรณ</t>
+  </si>
+  <si>
+    <t>เสาวลักษณ์กุล</t>
   </si>
 </sst>
 </file>
@@ -28094,7 +28100,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -28143,13 +28149,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="22"/>
+      </left>
+      <right style="thin">
+        <color indexed="22"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -28164,6 +28181,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -28446,7 +28469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3453"/>
+  <dimension ref="A1:G3455"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
@@ -107876,6 +107899,32 @@
       <c r="G3453" t="s">
         <v>9162</v>
       </c>
+    </row>
+    <row r="3454" spans="1:7">
+      <c r="A3454">
+        <v>6930104591</v>
+      </c>
+      <c r="B3454" t="s">
+        <v>9148</v>
+      </c>
+      <c r="C3454" s="8" t="s">
+        <v>9326</v>
+      </c>
+      <c r="D3454" s="8" t="s">
+        <v>9327</v>
+      </c>
+      <c r="E3454" s="8" t="s">
+        <v>970</v>
+      </c>
+      <c r="F3454" t="s">
+        <v>9157</v>
+      </c>
+      <c r="G3454" s="9" t="s">
+        <v>9154</v>
+      </c>
+    </row>
+    <row r="3455" spans="1:7">
+      <c r="F3455" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update staff database: add 3 new SAB68 advisors stably and improve staff parsing logic in convert_xlsx_to_js.py
</commit_message>
<xml_diff>
--- a/มอบตัว69 (1).xlsx
+++ b/มอบตัว69 (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\โครงการทิศทางเฟรชชี่ The Freshy Bearing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37EC04E0-8EC1-43AF-ADB9-020B959F7671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A6B8D1-1018-4D60-A7DB-33A52C1EE342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="มามอบตัว" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24327" uniqueCount="9328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24341" uniqueCount="9338">
   <si>
     <t>id_student</t>
   </si>
@@ -28022,6 +28022,36 @@
   </si>
   <si>
     <t>เสาวลักษณ์กุล</t>
+  </si>
+  <si>
+    <t>นายวินย์สันต์ วินทชัย</t>
+  </si>
+  <si>
+    <t>sab68</t>
+  </si>
+  <si>
+    <t>วิน</t>
+  </si>
+  <si>
+    <t>นายก องค์การบริหาร องค์การนิสิต SAB68</t>
+  </si>
+  <si>
+    <t>นายน้ำพุ จันทะสอน</t>
+  </si>
+  <si>
+    <t>ต้า</t>
+  </si>
+  <si>
+    <t>รองนายกฝ่ายสื่อสารองค์กร SAB68</t>
+  </si>
+  <si>
+    <t>รองนายกฝ่ายกิจกรรมนิสิต SAB68</t>
+  </si>
+  <si>
+    <t>น.ส.อาริศรา อุ่นอก</t>
+  </si>
+  <si>
+    <t>พิม</t>
   </si>
 </sst>
 </file>
@@ -28031,7 +28061,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28084,6 +28114,13 @@
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="TH SarabunPSK"/>
+      <family val="2"/>
+      <charset val="222"/>
     </font>
   </fonts>
   <fills count="3">
@@ -28166,7 +28203,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -28181,12 +28218,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -107933,7 +107971,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5005E9B0-F383-462D-BF33-F8893138837C}">
-  <dimension ref="A1:G112"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="22.2"/>
   <cols>
     <col min="1" max="1" width="10" style="4" bestFit="1" customWidth="1"/>
@@ -107942,7 +107980,9 @@
     <col min="5" max="5" width="11.88671875" style="4" customWidth="1"/>
     <col min="6" max="6" width="12.77734375" style="4" customWidth="1"/>
     <col min="7" max="7" width="16.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="4"/>
+    <col min="8" max="9" width="8.88671875" style="4"/>
+    <col min="10" max="10" width="20.33203125" style="4" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -108771,6 +108811,63 @@
       </c>
       <c r="G112" s="4" t="s">
         <v>9323</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7">
+      <c r="A114" s="4" t="s">
+        <v>9331</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7">
+      <c r="A115" s="4" t="s">
+        <v>9328</v>
+      </c>
+      <c r="E115" s="4" t="s">
+        <v>9222</v>
+      </c>
+      <c r="F115" s="4" t="s">
+        <v>9330</v>
+      </c>
+      <c r="G115" s="10">
+        <v>6530151494</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7">
+      <c r="A117" s="4" t="s">
+        <v>9335</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7">
+      <c r="A118" s="4" t="s">
+        <v>9332</v>
+      </c>
+      <c r="E118" s="4" t="s">
+        <v>9222</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>9333</v>
+      </c>
+      <c r="G118" s="4" t="s">
+        <v>9329</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7">
+      <c r="A120" s="4" t="s">
+        <v>9334</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7">
+      <c r="A121" s="4" t="s">
+        <v>9336</v>
+      </c>
+      <c r="E121" s="4" t="s">
+        <v>9222</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>9337</v>
+      </c>
+      <c r="G121" s="4" t="s">
+        <v>9329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>